<commit_message>
EPBDS-14346 Fix conversion when the argument type is String
</commit_message>
<xml_diff>
--- a/WSFrontend/org.openl.rules.ruleservice/test-resources/RulesFrontendTest/RulesFrontendTest/multimodule/Module3_1.xlsx
+++ b/WSFrontend/org.openl.rules.ruleservice/test-resources/RulesFrontendTest/RulesFrontendTest/multimodule/Module3_1.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="24">
   <si>
     <t>Method String worldHello(int hour)</t>
   </si>
@@ -62,6 +62,9 @@
   </si>
   <si>
     <t>return data;</t>
+  </si>
+  <si>
+    <t>Method String str2str(String data)</t>
   </si>
   <si>
     <t>Datatype Complex</t>
@@ -1410,7 +1413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="8.85156" style="1" customWidth="1"/>
@@ -1677,44 +1680,34 @@
     </row>
     <row r="32" ht="13.55" customHeight="1">
       <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
     </row>
     <row r="33" ht="13.55" customHeight="1">
-      <c r="A33" s="2"/>
-      <c r="B33" t="s" s="13">
+      <c r="A33" s="4"/>
+      <c r="B33" t="s" s="5">
         <v>17</v>
       </c>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="7"/>
       <c r="E33" s="2"/>
     </row>
     <row r="34" ht="13.55" customHeight="1">
-      <c r="A34" s="2"/>
-      <c r="B34" t="s" s="13">
-        <v>18</v>
-      </c>
-      <c r="C34" t="s" s="13">
-        <v>19</v>
-      </c>
-      <c r="D34" t="s" s="13">
-        <v>20</v>
-      </c>
+      <c r="A34" s="4"/>
+      <c r="B34" t="s" s="8">
+        <v>16</v>
+      </c>
+      <c r="C34" s="9"/>
+      <c r="D34" s="7"/>
       <c r="E34" s="2"/>
     </row>
     <row r="35" ht="13.55" customHeight="1">
       <c r="A35" s="2"/>
-      <c r="B35" t="s" s="13">
-        <v>21</v>
-      </c>
-      <c r="C35" t="s" s="13">
-        <v>22</v>
-      </c>
-      <c r="D35" s="14">
-        <v>25</v>
-      </c>
+      <c r="B35" s="10"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="2"/>
       <c r="E35" s="2"/>
     </row>
     <row r="36" ht="13.55" customHeight="1">
@@ -1724,8 +1717,50 @@
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
     </row>
+    <row r="37" ht="13.55" customHeight="1">
+      <c r="A37" s="2"/>
+      <c r="B37" t="s" s="13">
+        <v>18</v>
+      </c>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+    </row>
+    <row r="38" ht="13.55" customHeight="1">
+      <c r="A38" s="2"/>
+      <c r="B38" t="s" s="13">
+        <v>19</v>
+      </c>
+      <c r="C38" t="s" s="13">
+        <v>20</v>
+      </c>
+      <c r="D38" t="s" s="13">
+        <v>21</v>
+      </c>
+      <c r="E38" s="2"/>
+    </row>
+    <row r="39" ht="13.55" customHeight="1">
+      <c r="A39" s="2"/>
+      <c r="B39" t="s" s="13">
+        <v>22</v>
+      </c>
+      <c r="C39" t="s" s="13">
+        <v>23</v>
+      </c>
+      <c r="D39" s="14">
+        <v>25</v>
+      </c>
+      <c r="E39" s="2"/>
+    </row>
+    <row r="40" ht="13.55" customHeight="1">
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="17">
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B9:C9"/>
@@ -1741,6 +1776,8 @@
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>